<commit_message>
fixed current amps bug
</commit_message>
<xml_diff>
--- a/tests/coil_2D/input_template.xlsx
+++ b/tests/coil_2D/input_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="element_types"/>
@@ -368,7 +368,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -379,12 +379,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -416,7 +410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -447,12 +441,6 @@
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -759,16 +747,16 @@
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="12" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="13.290714285714287" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="6" width="14.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
     <col min="7" max="7" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>104</v>
       </c>
@@ -791,7 +779,7 @@
         <v>110</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1">
         <v>21</v>
       </c>
@@ -814,7 +802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1">
         <v>23</v>
       </c>
@@ -837,7 +825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1">
         <v>24</v>
       </c>
@@ -860,12 +848,12 @@
         <v>0</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="11"/>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+      <c r="A5" s="1"/>
       <c r="B5" s="3"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
     </row>
@@ -1478,7 +1466,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C2" s="1">
         <v>0</v>

</xml_diff>

<commit_message>
coil noint 2d tests
</commit_message>
<xml_diff>
--- a/tests/coil_2D/input_template.xlsx
+++ b/tests/coil_2D/input_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="4"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="element_types"/>
@@ -1335,7 +1335,7 @@
         <v>1e-8</v>
       </c>
       <c r="G4" s="9">
-        <v>8</v>
+        <v>1e-8</v>
       </c>
       <c r="H4" s="9">
         <v>0</v>

</xml_diff>